<commit_message>
refonte de la classe option, definition des grecs par différences finies, cleaning des jupyter
</commit_message>
<xml_diff>
--- a/Data for python project.xlsx
+++ b/Data for python project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sachamace/PycharmProjects/PythonProject2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51779815-AA30-3B4E-9EAE-FFDE0B1D428E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBB5B8BA-C95F-EA41-87B2-13D0D741E72D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15860" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -339,13 +339,13 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -586,6 +586,99 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>32356</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>604746</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>152076</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Image 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{202F6B33-A994-D843-81CF-224DE36A98B9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2046560" y="0"/>
+          <a:ext cx="5943600" cy="5588000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>647134</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>8089</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>56220</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>133067</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Image 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0B53A957-A4A1-0547-8EA9-2545D500155D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4675542" y="202229"/>
+          <a:ext cx="6794500" cy="3619500"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1846,7 +1939,7 @@
         <v>0.25</v>
       </c>
       <c r="B2" s="4">
-        <v>2.5899999999999999E-2</v>
+        <v>2.103E-2</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
@@ -1854,175 +1947,135 @@
         <v>0.5</v>
       </c>
       <c r="B3" s="4">
-        <v>2.5100000000000001E-2</v>
+        <v>2.4580000000000001E-2</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" s="2">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="B4" s="4">
-        <v>2.4899999999999999E-2</v>
+        <v>2.3900000000000001E-2</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" s="2">
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="B5" s="4">
-        <v>2.3900000000000001E-2</v>
+        <v>2.3099999999999999E-2</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" s="2">
-        <v>1.25</v>
+        <v>1.5</v>
       </c>
       <c r="B6" s="4">
-        <v>2.3099999999999999E-2</v>
+        <v>2.24E-2</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" s="2">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="B7" s="4">
-        <v>2.24E-2</v>
+        <v>2.8400000000000002E-2</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B8" s="4">
-        <v>2.4500000000000001E-2</v>
+        <v>2.93E-2</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B9" s="4">
-        <v>2.3800000000000002E-2</v>
+        <v>3.0300000000000001E-2</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" s="2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B10" s="4">
-        <v>2.35E-2</v>
+        <v>3.15E-2</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" s="2">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B11" s="4">
-        <v>2.3599999999999999E-2</v>
+        <v>3.2899999999999999E-2</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" s="2">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B12" s="4">
-        <v>2.3800000000000002E-2</v>
+        <v>3.4099999999999998E-2</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" s="2">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B13" s="4">
-        <v>2.4E-2</v>
+        <v>3.5499999999999997E-2</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" s="2">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B14" s="4">
-        <v>2.4299999999999999E-2</v>
+        <v>3.7699999999999997E-2</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" s="2">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B15" s="4">
-        <v>2.46E-2</v>
+        <v>3.9399999999999998E-2</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" s="2">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="B16" s="4">
-        <v>2.4899999999999999E-2</v>
+        <v>4.0800000000000003E-2</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" s="2">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="B17" s="4">
-        <v>2.52E-2</v>
+        <v>4.24E-2</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" s="2">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="B18" s="4">
-        <v>2.5399999999999999E-2</v>
+        <v>4.6699999999999998E-2</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" s="2">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="B19" s="4">
-        <v>2.5999999999999999E-2</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A20" s="2">
-        <v>20</v>
-      </c>
-      <c r="B20" s="4">
-        <v>2.6499999999999999E-2</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A21" s="2">
-        <v>25</v>
-      </c>
-      <c r="B21" s="4">
-        <v>2.6599999999999999E-2</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A22" s="2">
-        <v>30</v>
-      </c>
-      <c r="B22" s="4">
-        <v>2.6700000000000002E-2</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A23" s="2">
-        <v>40</v>
-      </c>
-      <c r="B23" s="4">
-        <v>2.6499999999999999E-2</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A24" s="2">
-        <v>50</v>
-      </c>
-      <c r="B24" s="4">
-        <v>2.6100000000000002E-2</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.2">
@@ -2220,6 +2273,7 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>